<commit_message>
Update published master datasets (2026-10-10)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -515,10 +515,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -11065,7 +11065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11838,26 +11838,26 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FOAK Builder: Programme Entry Expression of Interest</t>
+          <t>BridgeAI Deployment Catalyst: AI for Assurance and Compliance</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2600/overview/0c422454-a8af-4c24-a74a-565426f42395</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-assurance-and-compliance/</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026-10-07 17:10</t>
+          <t>2026-10-10 15:37</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>46302.71527777778</v>
+        <v>46305.65069444444</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -11866,19 +11866,25 @@
       <c r="H14" t="b">
         <v>0</v>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>46316</v>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Thursday 5 November 2026 11:00am</t>
+          <t>08/12/2026                              11:00</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>46331.45833333334</v>
+        <v>46364.45833333334</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>£100.0 million</t>
+          <t>£52.0 million</t>
         </is>
       </c>
       <c r="N14" s="2" t="n">
@@ -11891,26 +11897,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 10</t>
+          <t>BridgeAI Deployment Catalyst: AI for Decision Critical Systems</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2596/overview/31f0a768-2a9a-405d-b0a4-83a8c5b395c0</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-decision-critical-systems/</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-08 17:07</t>
+          <t>2026-10-10 15:37</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>46303.71319444444</v>
+        <v>46305.65069444444</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -11919,25 +11925,196 @@
       <c r="H15" t="b">
         <v>0</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>46316</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
+          <t>08/12/2026                              11:00</t>
         </is>
       </c>
       <c r="L15" s="2" t="n">
-        <v>46358.45833333334</v>
+        <v>46364.45833333334</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£52.0 million</t>
         </is>
       </c>
       <c r="N15" s="2" t="n">
         <v>46302</v>
       </c>
       <c r="O15" s="1" t="n">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BridgeAI Deployment Catalyst: AI for Operational Systems</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/bridgeai-deployment-catalyst-ai-for-operational-systems/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:37</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>46305.65069444444</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>08/12/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="n">
+        <v>46364.45833333334</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>£52.0 million</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FOAK Builder: Programme Entry Expression of Interest</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2600/overview/0c422454-a8af-4c24-a74a-565426f42395</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-10-07 17:10</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>46302.71527777778</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Thursday 5 November 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="n">
+        <v>46331.45833333334</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>£100.0 million</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O17" s="1" t="n">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Full ADOPT Grant: Round 10</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2596/overview/31f0a768-2a9a-405d-b0a4-83a8c5b395c0</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:07</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>46303.71319444444</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>£200,000</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O18" s="1" t="n">
         <v>46302</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-12)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -515,10 +515,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -11065,7 +11065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12015,26 +12015,26 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FOAK Builder: Programme Entry Expression of Interest</t>
+          <t>HMGCC Co-Creation Challenge: Smart glasses for mapping</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2600/overview/0c422454-a8af-4c24-a74a-565426f42395</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-smart-glasses-for-mapping/</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-10-07 17:10</t>
+          <t>2026-10-12 19:27</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>46302.71527777778</v>
+        <v>46307.81041666667</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
@@ -12043,19 +12043,23 @@
       <c r="H17" t="b">
         <v>0</v>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>46307</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Thursday 5 November 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="n">
-        <v>46331.45833333334</v>
-      </c>
+          <t>12/11/2026</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
-          <t>£100.0 million</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N17" s="2" t="n">
@@ -12068,26 +12072,26 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 10</t>
+          <t>HMGCC Co-Creation Challenge: Multi-Terrain Micro Robotic Systems</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2596/overview/31f0a768-2a9a-405d-b0a4-83a8c5b395c0</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/hmgcc-co-creation-challenge-multi-terrain-micro-robotic-systems/</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-08 17:07</t>
+          <t>2026-10-12 19:27</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>46303.71319444444</v>
+        <v>46307.81041666667</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -12096,25 +12100,135 @@
       <c r="H18" t="b">
         <v>0</v>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>46307</v>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="n">
-        <v>46358.45833333334</v>
-      </c>
+          <t>12/11/2026</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£60,000</t>
         </is>
       </c>
       <c r="N18" s="2" t="n">
         <v>46302</v>
       </c>
       <c r="O18" s="1" t="n">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FOAK Builder: Programme Entry Expression of Interest</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2600/overview/0c422454-a8af-4c24-a74a-565426f42395</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-10-07 17:10</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>46302.71527777778</v>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Thursday 5 November 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>46331.45833333334</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>£100.0 million</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Full ADOPT Grant: Round 10</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2596/overview/31f0a768-2a9a-405d-b0a4-83a8c5b395c0</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-10-08 17:07</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>46303.71319444444</v>
+      </c>
+      <c r="F20" t="b">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>£200,000</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O20" s="1" t="n">
         <v>46302</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-15)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -516,10 +516,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -11212,7 +11212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11295,26 +11295,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+          <t>European Space Agency: Space-Enabled Solutions For Resilient Grids</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/european-space-agency-space-enabled-solutions-for-resilient-grids/</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-14 14:50</t>
+          <t>2026-10-15 14:30</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>46309.61805555555</v>
+        <v>46310.60416666666</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -11323,25 +11323,137 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>02/11/2026</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>46328</v>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>46358.45833333334</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>£54,400</t>
-        </is>
-      </c>
+          <t>29/01/2027</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" s="2" t="n">
         <v>46309</v>
       </c>
       <c r="O2" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Growth Cohorts: Next generation low carbon concrete</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/growth-cohorts-next-generation-low-carbon-concrete/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:30</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>46310.60416666666</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>02/12/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>£11.5 million</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:50</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>46309.61805555555</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>£54,400</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O4" s="1" t="n">
         <v>46309</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-19)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -513,13 +513,13 @@
         <v>46309</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -11212,7 +11212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11407,26 +11407,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+          <t>UK Defence Innovation: Tactical Power Challenge</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/uk-defence-innovation-tactical-power-challenge/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-10-14 14:50</t>
+          <t>2026-10-19 16:39</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>46309.61805555555</v>
+        <v>46314.69375</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -11435,25 +11435,243 @@
       <c r="H4" t="b">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>46311</v>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
+          <t>10/11/2026                              12:00</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>46358.45833333334</v>
+        <v>46336.5</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>£54,400</t>
+          <t>£2.5 million</t>
         </is>
       </c>
       <c r="N4" s="2" t="n">
         <v>46309</v>
       </c>
       <c r="O4" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EIT Culture &amp; Creativity: New Ventures in Creative Tech (Spark Incubation)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/eit-culture-creativity-new-ventures-in-creative-tech-spark-incubation/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:39</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>46314.69375</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>16/11/2026</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O5" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>What Works Centre for a climate resilient UK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/what-works-centre-for-a-climate-resilient-uk/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:39</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46314.69375</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>15/12/2026</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>£21.1 million</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O6" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:50</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46309.61805555555</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>£54,400</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O7" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Knowledge Transfer Partnership (KTP): 2026 - 2027 Round 4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2605/overview/4b82d27a-2794-457c-8dc7-7ec4f6911c84</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:45</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>46314.69791666666</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Wednesday 27 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>46414.45833333334</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O8" s="1" t="n">
         <v>46309</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-20)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -516,10 +516,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -11212,7 +11212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11576,26 +11576,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+          <t>Knowledge Transfer Partnership (KTP): 2026 - 2027 Round 4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/knowledge-transfer-partnership-ktp-2026-2027-round-4/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-14 14:50</t>
+          <t>2026-10-20 14:32</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>46309.61805555555</v>
+        <v>46315.60555555556</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -11604,19 +11604,25 @@
       <c r="H7" t="b">
         <v>0</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>46314</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Wednesday 2 December 2026 11:00am</t>
+          <t>27/01/2027                              11:00</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>46358.45833333334</v>
+        <v>46414.45833333334</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>£54,400</t>
+          <t>£12.5 million</t>
         </is>
       </c>
       <c r="N7" s="2" t="n">
@@ -11629,26 +11635,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2026 - 2027 Round 4</t>
+          <t>iX Challenge: Smart control solutions for domestic hybrid heating systems</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2605/overview/4b82d27a-2794-457c-8dc7-7ec4f6911c84</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-smart-control-solutions-for-domestic-hybrid-heating-systems/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-19 16:45</t>
+          <t>2026-10-20 14:32</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46314.69791666666</v>
+        <v>46315.60555555556</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -11657,21 +11663,182 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>46315</v>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Wednesday 27 January 2027 11:00am</t>
+          <t>01/12/2026                              11:59</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
-        <v>46414.45833333334</v>
+        <v>46357.49930555555</v>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" s="2" t="n">
         <v>46309</v>
       </c>
       <c r="O8" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>iX Challenge: Developing cost-effective polyols from UK waste-carbon for digital mass manufacturing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-developing-cost-effective-polyols-from-uk-waste-carbon/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:32</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>46315.60555555556</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Growth Cohorts: Next-gen low carbon concrete cohort entry Round 2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2602/overview/607351e2-798f-450b-b77d-3131912bcbef</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:50</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>46309.61805555555</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Wednesday 2 December 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>46358.45833333334</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>£54,400</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Knowledge Transfer Partnership (KTP): 2026 - 2027 Round 4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2605/overview/4b82d27a-2794-457c-8dc7-7ec4f6911c84</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:45</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46314.69791666666</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Wednesday 27 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>46414.45833333334</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O11" s="1" t="n">
         <v>46309</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-23)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -517,10 +517,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -11669,7 +11669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11919,26 +11919,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Healthy Soils and Water for a Sustainable Environment</t>
+          <t>Secure Innovation Security Reviews</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/secure-innovation-security-review/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-10-22 14:49</t>
+          <t>2026-10-23 14:29</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>46317.61736111111</v>
+        <v>46318.60347222222</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -11947,25 +11947,84 @@
       <c r="H5" t="b">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>46318</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Thursday 28 January 2027 11:00am</t>
+          <t>31/01/2027                              12:00</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>46415.45833333334</v>
+        <v>46418.5</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£315,000</t>
         </is>
       </c>
       <c r="N5" s="2" t="n">
         <v>46316</v>
       </c>
       <c r="O5" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:49</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>46317.61736111111</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Thursday 28 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>46415.45833333334</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>£5.0 million</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O6" s="1" t="n">
         <v>46316</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-24)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -517,10 +517,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -11669,7 +11669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11978,26 +11978,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Healthy Soils and Water for a Sustainable Environment</t>
+          <t>iX Challenge: Systemic capture and analysis of structural condition data</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-systemic-capture-and-analysis-of-structural-condition-data/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-10-22 14:49</t>
+          <t>2026-10-24 13:41</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>46317.61736111111</v>
+        <v>46319.57013888889</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -12006,25 +12006,78 @@
       <c r="H6" t="b">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>46318</v>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Thursday 28 January 2027 11:00am</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>46415.45833333334</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>£5.0 million</t>
-        </is>
-      </c>
+          <t>04/12/2026</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" s="2" t="n">
         <v>46316</v>
       </c>
       <c r="O6" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:49</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>46317.61736111111</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Thursday 28 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>46415.45833333334</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>£5.0 million</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O7" s="1" t="n">
         <v>46316</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update published master datasets (2026-10-27)
</commit_message>
<xml_diff>
--- a/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
+++ b/outputs/InnovateUK_Funding_Opportunities_WeeklyBreakdown.xlsx
@@ -517,10 +517,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -11669,7 +11669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12031,26 +12031,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Healthy Soils and Water for a Sustainable Environment</t>
+          <t>EIT Health: Innovation Validation Call 2027</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/eit-health-innovation-validation-call-2027/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-10-22 14:49</t>
+          <t>2026-10-27 15:34</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>46317.61736111111</v>
+        <v>46322.64861111111</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -12059,21 +12059,21 @@
       <c r="H7" t="b">
         <v>0</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>46309</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Thursday 28 January 2027 11:00am</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>46415.45833333334</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>£5.0 million</t>
-        </is>
-      </c>
+          <t>13/01/2027</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" s="2" t="n">
         <v>46316</v>
       </c>
@@ -12084,26 +12084,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Underground hydrogen storage demonstrator DEVEX support</t>
+          <t>Testing and validating underground hydrogen storage components</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2608/overview/edd17e49-cb74-4ae3-89ee-0ceed80c4618</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/testing-and-validating-underground-hydrogen-storage-components/</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-10-26 16:25</t>
+          <t>2026-10-27 15:34</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>46321.68402777778</v>
+        <v>46322.64861111111</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -12112,11 +12112,17 @@
       <c r="H8" t="b">
         <v>0</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>46318</v>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Wednesday 13 January 2027 11:00am</t>
+          <t>13/01/2027                              11:00</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
@@ -12124,7 +12130,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>£750,000</t>
+          <t>£28.0 million</t>
         </is>
       </c>
       <c r="N8" s="2" t="n">
@@ -12137,26 +12143,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Testing and validating underground hydrogen storage components</t>
+          <t>Underground hydrogen storage demonstrator DEVEX support</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2606/overview/52a725a1-ecfe-4eec-a30a-ac6d4078c350</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/underground-hydrogen-storage-demonstrator-devex-support/</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-10-26 16:25</t>
+          <t>2026-10-27 15:34</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>46321.68402777778</v>
+        <v>46322.64861111111</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -12165,11 +12171,17 @@
       <c r="H9" t="b">
         <v>0</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>46318</v>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Wednesday 13 January 2027 11:00am</t>
+          <t>13/01/2027                              11:00</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
@@ -12177,13 +12189,231 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£28.0 million</t>
         </is>
       </c>
       <c r="N9" s="2" t="n">
         <v>46316</v>
       </c>
       <c r="O9" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/healthy-soils-and-water-for-a-sustainable-environment/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-10-27 15:34</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>46322.64861111111</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>19/11/2026</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>46345</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>28/01/2027                              11:00</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>46415.45833333334</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>£28.0 million</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Healthy Soils and Water for a Sustainable Environment</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2604/overview/0a26a044-e3c5-4fa0-8556-b382497374df</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:49</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>46317.61736111111</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Thursday 28 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>46415.45833333334</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>£5.0 million</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Underground hydrogen storage demonstrator DEVEX support</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2608/overview/edd17e49-cb74-4ae3-89ee-0ceed80c4618</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:25</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>46321.68402777778</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Wednesday 13 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>46400.45833333334</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>£750,000</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Testing and validating underground hydrogen storage components</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2606/overview/52a725a1-ecfe-4eec-a30a-ac6d4078c350</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:25</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>46321.68402777778</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Wednesday 13 January 2027 11:00am</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>46400.45833333334</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>£5.0 million</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="O13" s="1" t="n">
         <v>46316</v>
       </c>
     </row>

</xml_diff>